<commit_message>
Tell operators what every GD line needs
</commit_message>
<xml_diff>
--- a/myapp-frontend/public/templates/gd-costing-template.xlsx
+++ b/myapp-frontend/public/templates/gd-costing-template.xlsx
@@ -1306,7 +1306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1568,12 +1568,26 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">  4. A row with no HS code still imports - it is just not classified.</t>
+          <t xml:space="preserve">  4. Every row needs its GD Date, HS Code, Unit and an Assessed Value above</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     zero, and its Unit must be the one the item is kept in. A row missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     one is shown in the preview to fix; it cannot come in until it is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t xml:space="preserve">  5. Headings live on row 1 and data starts on row 3. Do not delete row 2.</t>
         </is>

</xml_diff>